<commit_message>
feat(excel): update sample enrollments spreadsheet with 6 workshops and edge test cases
</commit_message>
<xml_diff>
--- a/SkillHub.Web/wwwroot/sample_enrollments.xlsx
+++ b/SkillHub.Web/wwwroot/sample_enrollments.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -26,7 +26,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>maria.rodriguez@example.com</t>
+          <t>juan.perez@example.com</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -38,60 +38,192 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>pedro.gomez@example.com</t>
+          <t>maria.rodriguez@example.com</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>COC-001</t>
+          <t>FOT-001</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ana.martinez@example.com</t>
+          <t>carlos.lopez@example.com</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ORA-001</t>
+          <t>COC-001</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>maria.rodriguez@example.com</t>
+          <t>ana.martinez@example.com</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>COC-001</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>noexiste@correo.com</t>
+          <t>camila.cardenas@correo.com</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FOT-001</t>
+          <t>ORA-001</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>pedro.gomez@example.com</t>
+          <t>felipe.agudelo@correo.com</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>INEXISTENTE-999</t>
+          <t>ORA-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>daniela.morales@correo.com</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DIS-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>santiago.ramirez@correo.com</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DIS-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>valentina.gomez@correo.com</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MAT-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>andres.salazar@correo.com</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MAT-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>laura.martinez@correo.com</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MUS-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>diego.munoz@correo.com</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MUS-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>juan.perez@example.com</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MUS-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>maria.rodriguez@example.com</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MAT-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>juan.perez@example.com</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FOT-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>usuario.no.registrado@correo.com</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>COC-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>carlos.lopez@example.com</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TALLER-999</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(excel): add dedicated workshops excel spreadsheet and update import UI
</commit_message>
<xml_diff>
--- a/SkillHub.Web/wwwroot/sample_enrollments.xlsx
+++ b/SkillHub.Web/wwwroot/sample_enrollments.xlsx
@@ -2,13 +2,317 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Enrollments" sheetId="1" r:id="rId1"/>
+    <sheet name="Workshops" sheetId="1" r:id="rId1"/>
+    <sheet name="Enrollments" sheetId="2" r:id="rId2"/>
+    <sheet name="Instructors" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>InstructorEmail</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>InstructorName</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>StartDate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>EndDate</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FOT-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fotografía Urbana y Manejo de Luz Natural</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Taller práctico sobre composición visual, captura callejera y aprovechamiento de luz ambiental.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>carlos.mendoza@skillhub.com</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Carlos Mendoza</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-11-03 09:00</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-11-03 13:00</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>COC-001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cocina Mediterránea Básica</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Aprende técnicas fundamentales de preparación, pastas frescas y salsas clásicas.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>laura.gomez@skillhub.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Laura Gómez</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-11-04 14:00</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-11-04 18:00</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ORA-001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Oratoria y Comunicación Asertiva</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Técnicas de modulación de voz, lenguaje no verbal y persuasión para hablar en público con confianza.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>andres.torres@skillhub.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Andrés Torres</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-11-05 10:00</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-11-05 14:00</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DIS-001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Fundamentos de Diseño Visual y Branding</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Creación de identidades de marca, teoría del color, tipografía y diseño con propósito.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>sofia.morales@skillhub.com</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sofía Morales</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-11-06 15:00</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-11-06 19:00</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MAT-001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Matemáticas Básicas y Aplicadas</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Aprende matemáticas y resolución de problemas prácticos.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>andres.torres@skillhub.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Andrés Torres</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-11-25 10:00</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-11-25 13:00</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MUS-001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Guitarra desde cero</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Acordes básicos y primeras canciones.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>hernan.quintero@correo.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Hernán Darío Quintero Gil</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-12-12 19:00</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-12-12 22:00</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:B18"/>
   <sheetData>
     <row r="1">
@@ -229,4 +533,131 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>FullName</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Specialty</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Carlos Mendoza</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>carlos.mendoza@skillhub.com</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Fotografía</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Laura Gómez</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>laura.gomez@skillhub.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Andrés Torres</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>andres.torres@skillhub.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Oratoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sofía Morales</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sofia.morales@skillhub.com</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Diseño Gráfico</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Hernán Darío Quintero Gil</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>hernan.quintero@correo.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Música</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Admin SkillHub</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>admin@skillhub.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Coordinación</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>